<commit_message>
Update budget (new controller)
</commit_message>
<xml_diff>
--- a/random-managerial-stuff/budget.xlsx
+++ b/random-managerial-stuff/budget.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Item</t>
   </si>
@@ -22,19 +27,19 @@
     <t>Link</t>
   </si>
   <si>
-    <t>Stepper Motor driver</t>
+    <t xml:space="preserve">Stepper Motor driver</t>
   </si>
   <si>
     <t>https://www.amazon.co.uk/gp/product/B081JM828X?smid=A3SCFTIO8CSK1X&amp;psc=1</t>
   </si>
   <si>
-    <t>Idler (toothed)</t>
+    <t xml:space="preserve">Idler (toothed)</t>
   </si>
   <si>
     <t>https://www.amazon.co.uk/Printer-Idler-Pulley-Toothed-Smooth/dp/B075GPMB8T?crid=2C14GCF9ZSSWM&amp;dib=eyJ2IjoiMSJ9.z9_KOU9R-x4VTuzAk1MUF3FjAQSMLjsG7UDRNxnXtNVwSKC1MkP5A44VnFcicTELOoO5HGJ1HkuqebkJrLUDNZXEm93Tt5w78OMDZ4rMZsB-YPMOKv_PHAPAdEpnQnf5SpnczGZIOEb1ccsDMJuURe_ytzoAXyoLRfPwAiOPJbTUgMNOnc6fVJFpFS6UTcoFaIRDsx2WG_KDi0iuFdP5IkbGiqPRmIBWdkoXuFOWes_kumI0CD3gOGPo_HGKcwTbiOzRQYeQ_3GqSuJmOwau-HONd-7ImctEqyFL8EbpgaE.ZDz2YWB9TRvYD6LwLGCGU6-dnQtQ5xNAU_3AVaJFL00&amp;dib_tag=se&amp;keywords=6mm%2Bwide%2Bbelt%2Bidler%2Bpulley&amp;qid=1772494539&amp;s=industrial&amp;sprefix=6mm%2Bwide%2Bbelt%2Bidler%2Bpulle%2Cindustrial%2C214&amp;sr=1-18&amp;th=1</t>
   </si>
   <si>
-    <t>Idler (smooth)</t>
+    <t xml:space="preserve">Idler (smooth)</t>
   </si>
   <si>
     <t>Rods</t>
@@ -43,7 +48,7 @@
     <t>https://botland.store/components-for-3d-printers-construction/18918-linear-shaft-8mm-length-350mm-5904422354879.html</t>
   </si>
   <si>
-    <t>Timing belt + pulleys</t>
+    <t xml:space="preserve">Timing belt + pulleys</t>
   </si>
   <si>
     <t>https://www.amazon.co.uk/JZK-Meters-timing-pulley-printer/dp/B094YBZJG8?crid=1RHDO4RFXREPC&amp;dib=eyJ2IjoiMSJ9.Bn85vzetQ8HkvitX1UStilcaw3X1XWvOAXTD8OG3LGpHDPeQor0vcON9oA21l4oLEC81ThJ_hwy1xPnUYW3qU-ROEeqAWk3YS402SEsI0eD8jbawOOOc87O4A8G75ULsk6K0SKPQUxSDA5P-jHXPpPy_1XFH5XgX0Dj0HKZMaAE0zV9gNUk0hjsrSZITBSdEOHeqytZONTToEAB1QBrGQcN0hKDkbhqU80DTmYcMIe_NoWuQV8zl1Jn2BrUkDtJVvKGrFlnRkYSyIU5ThHBoNdzv1BdFR33oU86-_c8CCa4.MKj4FTdjprEhVNXDkZRB0IkR7PCBG8dz4Zi-XDa_AU4&amp;dib_tag=se&amp;keywords=gt2+5mm+belt&amp;qid=1772494819&amp;s=industrial&amp;sprefix=gt2+5mm+belt%2Cindustrial%2C215&amp;sr=1-11</t>
@@ -61,10 +66,10 @@
     <t>https://ooznest.co.uk/product/mechanical-endstop/</t>
   </si>
   <si>
-    <t>CNCShield</t>
-  </si>
-  <si>
-    <t>https://www.ebay.co.uk/itm/356994873056?chn=ps&amp;_ul=GB&amp;google_free_listing_action=view_item</t>
+    <t>MotorController</t>
+  </si>
+  <si>
+    <t>https://www.ebay.co.uk/itm/406186602711?_ul=GB&amp;rb_itemId=406186602711&amp;rb_pgeo=GB&amp;toolid=10044&amp;var=0&amp;ff=11</t>
   </si>
   <si>
     <t>Stepper</t>
@@ -76,11 +81,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
+      <sz val="10.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -91,14 +96,16 @@
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <color indexed="4"/>
     </font>
     <font>
-      <color rgb="FF000000"/>
+      <color indexed="64"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
+      <sz val="10.000000"/>
+      <color theme="10"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -106,50 +113,337 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -206,7 +500,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -232,7 +526,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -309,7 +603,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -339,17 +633,19 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="12.63"/>
+    <col customWidth="1" min="2" max="2" width="12.630000000000001"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -368,7 +664,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>4</v>
@@ -379,7 +675,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
@@ -390,7 +686,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
@@ -401,7 +697,7 @@
         <v>8</v>
       </c>
       <c r="B6" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>9</v>
@@ -412,7 +708,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="1">
-        <v>8.49</v>
+        <v>8.4900000000000002</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -423,7 +719,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="1">
-        <v>6.99</v>
+        <v>6.9900000000000002</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>13</v>
@@ -434,9 +730,9 @@
         <v>8</v>
       </c>
       <c r="B9" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="C9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -445,7 +741,7 @@
         <v>14</v>
       </c>
       <c r="B10" s="1">
-        <v>1.62</v>
+        <v>1.6200000000000001</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>15</v>
@@ -456,9 +752,9 @@
         <v>14</v>
       </c>
       <c r="B11" s="1">
-        <v>1.62</v>
-      </c>
-      <c r="C11" s="4" t="s">
+        <v>1.6200000000000001</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -467,9 +763,9 @@
         <v>14</v>
       </c>
       <c r="B12" s="1">
-        <v>1.62</v>
-      </c>
-      <c r="C12" s="4" t="s">
+        <v>1.6200000000000001</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -478,9 +774,9 @@
         <v>14</v>
       </c>
       <c r="B13" s="1">
-        <v>1.62</v>
-      </c>
-      <c r="C13" s="4" t="s">
+        <v>1.6200000000000001</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -489,9 +785,9 @@
         <v>16</v>
       </c>
       <c r="B14" s="1">
-        <v>4.99</v>
-      </c>
-      <c r="C14" s="2" t="s">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -500,9 +796,9 @@
         <v>18</v>
       </c>
       <c r="B15" s="1">
-        <v>12.0</v>
-      </c>
-      <c r="C15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -511,7 +807,7 @@
         <v>18</v>
       </c>
       <c r="B16" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>19</v>
@@ -520,26 +816,29 @@
     <row r="17">
       <c r="B17" s="5">
         <f>SUM(B3:B16)</f>
-        <v>75.95</v>
+        <v>75.97999999999999</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C3"/>
     <hyperlink r:id="rId2" ref="C4"/>
-    <hyperlink r:id="rId3" ref="C5"/>
-    <hyperlink r:id="rId4" ref="C6"/>
-    <hyperlink r:id="rId5" ref="C7"/>
-    <hyperlink r:id="rId6" ref="C8"/>
-    <hyperlink r:id="rId7" ref="C9"/>
-    <hyperlink r:id="rId8" ref="C10"/>
-    <hyperlink r:id="rId9" ref="C11"/>
-    <hyperlink r:id="rId10" ref="C12"/>
-    <hyperlink r:id="rId11" ref="C13"/>
-    <hyperlink r:id="rId12" ref="C14"/>
-    <hyperlink r:id="rId13" ref="C15"/>
-    <hyperlink r:id="rId14" ref="C16"/>
+    <hyperlink r:id="rId2" ref="C5"/>
+    <hyperlink r:id="rId3" ref="C6"/>
+    <hyperlink r:id="rId4" ref="C7"/>
+    <hyperlink r:id="rId5" ref="C8"/>
+    <hyperlink r:id="rId3" ref="C9"/>
+    <hyperlink r:id="rId6" ref="C10"/>
+    <hyperlink r:id="rId6" ref="C11"/>
+    <hyperlink r:id="rId6" ref="C12"/>
+    <hyperlink r:id="rId6" ref="C13"/>
+    <hyperlink r:id="rId7" ref="C14"/>
+    <hyperlink r:id="rId8" ref="C15"/>
+    <hyperlink r:id="rId8" ref="C16"/>
   </hyperlinks>
-  <drawing r:id="rId15"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>